<commit_message>
Update text to "Possible duplicate lines"
</commit_message>
<xml_diff>
--- a/1-stress-test/test-results/paddle_vs_abbyy_errors_artifacts.xlsx
+++ b/1-stress-test/test-results/paddle_vs_abbyy_errors_artifacts.xlsx
@@ -42,10 +42,10 @@
     <t>reading order - abbyy</t>
   </si>
   <si>
-    <t>duplicate/tile overlap - paddle</t>
-  </si>
-  <si>
-    <t>duplicate/tile overlap - abbyy</t>
+    <t>Possible duplicate lines - paddle</t>
+  </si>
+  <si>
+    <t>Possible duplicate lines - abbyy</t>
   </si>
   <si>
     <t>OCR token/phrase mismatch - paddle</t>
@@ -390,7 +390,7 @@
     <t>L960: abbreviation/spacing may be garbled :: Captain A.H.Bogardus, of Elkhart, ., Ill.,</t>
   </si>
   <si>
-    <t>duplicate/tile overlap issue count</t>
+    <t>Possible duplicate lines issue count</t>
   </si>
   <si>
     <t>4</t>

</xml_diff>